<commit_message>
Update charts and table, also modify description of instance types
</commit_message>
<xml_diff>
--- a/collected_results/Summary_Result.xlsx
+++ b/collected_results/Summary_Result.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9baf9ac8cfa6ebe3/文件/2025-26 semester B/CS4296/group project/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9baf9ac8cfa6ebe3/文件/2025-26 semester B/CS4296/group project/Test_Result/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="120" documentId="8_{5F421939-039C-425A-9A0B-C3D8730F6B95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7D8F1AB7-A4DB-4A6D-AF1F-EB8C770FD1F7}"/>
+  <xr:revisionPtr revIDLastSave="149" documentId="8_{5F421939-039C-425A-9A0B-C3D8730F6B95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D00801A0-F3B0-44CF-B6D4-02ECA0045B89}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="20880" xr2:uid="{983D5BFB-60EB-4053-9114-F21B1579F0FD}"/>
+    <workbookView minimized="1" xWindow="15" yWindow="15" windowWidth="38370" windowHeight="20850" xr2:uid="{983D5BFB-60EB-4053-9114-F21B1579F0FD}"/>
   </bookViews>
   <sheets>
     <sheet name="工作表1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="23">
   <si>
     <t>Rank</t>
   </si>
@@ -109,12 +109,19 @@
     <t>(round to 4 significant figures)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
+  <si>
+    <t>Queries per $1 USD</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="177" formatCode="#,##0.00_ "/>
+  </numFmts>
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -146,6 +153,13 @@
       <b/>
       <sz val="12"/>
       <color rgb="FF0F1115"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
@@ -206,7 +220,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -226,6 +240,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -335,7 +358,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
                       <a:schemeClr val="tx1">
                         <a:lumMod val="75000"/>
@@ -479,7 +502,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -692,7 +715,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
                       <a:schemeClr val="tx1">
                         <a:lumMod val="75000"/>
@@ -836,7 +859,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -1060,7 +1083,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
                       <a:schemeClr val="tx1">
                         <a:lumMod val="75000"/>
@@ -1820,7 +1843,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
                       <a:schemeClr val="tx1">
                         <a:lumMod val="75000"/>
@@ -1964,7 +1987,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -2177,7 +2200,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
                       <a:schemeClr val="tx1">
                         <a:lumMod val="75000"/>
@@ -2321,7 +2344,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -2546,7 +2569,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
                       <a:schemeClr val="tx1">
                         <a:lumMod val="75000"/>
@@ -7052,7 +7075,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C874948-3DE1-4912-A02E-2B05BAD813AE}">
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.25" bestFit="1" customWidth="1"/>
@@ -7065,9 +7088,10 @@
     <col min="8" max="8" width="56.25" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="53.75" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="50.625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="23.625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>20</v>
       </c>
@@ -7083,7 +7107,7 @@
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
@@ -7099,23 +7123,26 @@
       <c r="E2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I2" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="J2" s="8" t="s">
         <v>19</v>
       </c>
+      <c r="K2" s="7" t="s">
+        <v>22</v>
+      </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -7146,8 +7173,12 @@
       <c r="J3" s="6">
         <v>0.126</v>
       </c>
+      <c r="K3" s="9">
+        <f>(E3*3600)/H3</f>
+        <v>12032307.692307692</v>
+      </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -7178,8 +7209,12 @@
       <c r="J4" s="6">
         <v>8.5000000000000006E-2</v>
       </c>
+      <c r="K4" s="9">
+        <f t="shared" ref="K4:K8" si="0">(E4*3600)/H4</f>
+        <v>17340674.157303371</v>
+      </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -7210,8 +7245,12 @@
       <c r="J5" s="6">
         <v>9.6000000000000002E-2</v>
       </c>
+      <c r="K5" s="9">
+        <f t="shared" si="0"/>
+        <v>14853600</v>
+      </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -7242,8 +7281,12 @@
       <c r="J6" s="6">
         <v>8.3199999999999996E-2</v>
       </c>
+      <c r="K6" s="9">
+        <f t="shared" si="0"/>
+        <v>15047750.865051903</v>
+      </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -7274,8 +7317,12 @@
       <c r="J7" s="6">
         <v>4.1599999999999998E-2</v>
       </c>
+      <c r="K7" s="9">
+        <f t="shared" si="0"/>
+        <v>26644789.356984477</v>
+      </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -7305,6 +7352,10 @@
       </c>
       <c r="J8" s="6">
         <v>1.04E-2</v>
+      </c>
+      <c r="K8" s="9">
+        <f t="shared" si="0"/>
+        <v>102224460.43165468</v>
       </c>
     </row>
   </sheetData>

</xml_diff>